<commit_message>
Final 5-run measured execution + reviewer fixes
- 5 complete end-to-end runs against real Anthropic API (/bin/zsh.43 total, /bin/zsh.086/run)
- Token Math Sheet populated with measured per-call costs in Column N + measured E/F token counts; projected annual at 750-account scale: ,361 vs k budget (~2.7%)
- AI Build Process Memo (.docx) finalised
- README expanded with measured evidence packet + known limitations (judge anchoring, 24/7 batch sim, hierarchical prio needed at scale) + model-ID note
- run_summary.json per run now includes failure_signals (parse errors, escalations, intervention triggers)
- Applied fixes from external code review (Codex gpt-5.5 + Gemini 3 Pro): stale docstrings, retry-count docstring alignment, judge anchoring caveat, telemetry-claim correction in routing.py

Repo public at https://github.com/dashunter-cloud/2hl-cs-workflow

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/AI_System_Design_Assessment_Token_Math_Sheet_DavidHunter.xlsx
+++ b/outputs/AI_System_Design_Assessment_Token_Math_Sheet_DavidHunter.xlsx
@@ -802,7 +802,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>A cost-tiered customer-success pipeline for a 750-account portfolio. Haiku handles the high-volume daily account scan and inbound ticket triage; Sonnet handles synthesis stages (prioritisation, check-in prep, quality review with an INDEPENDENT-CALL JUDGE for quality control); Opus is reserved for the bi-weekly segment-intervention design. Deterministic routing applies policy at the boundaries. The architecture is generator-plus-judge with calibration gates at each stage so failures are noisy (escalation) rather than quiet (drift). Same pattern I run in production at Kickstone (Sonny Jim, DISCOVER, KS Rapport).</t>
+          <t>Cost-tiered customer-success pipeline for a 750-account portfolio. Haiku 4.5 handles the high-volume daily account scan and inbound ticket triage. Sonnet 4.6 handles synthesis stages (portfolio prioritisation, check-in prep, quality-review generator). The quality-review JUDGE is a DIFFERENT MODEL (Haiku 4.5) - real discriminator separation, ~11x cheaper than the Sonnet generator, and cost-tier-correct because verification is simpler than synthesis. Opus 4.7 is reserved for bi-weekly segment-intervention design. Deterministic routing applies policy at the boundaries. Measured per-call costs (column N) come from a real 5-run end-to-end execution on the synthetic dataset; avg cost per end-to-end run is $0.086. Projected annual cost at 750-account scale: $1,361 - 2.7% of the $50k budget. Headroom for prompt caching, denser quality review, and richer memory retrieval at production scale.</t>
         </is>
       </c>
       <c r="F4" s="27" t="n"/>
@@ -1036,10 +1036,10 @@
         <v>750</v>
       </c>
       <c r="E12" s="35" t="n">
-        <v>1200</v>
+        <v>530</v>
       </c>
       <c r="F12" s="35" t="n">
-        <v>300</v>
+        <v>128</v>
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
@@ -1072,10 +1072,12 @@
         <f>IF(L12="","",L12*260)</f>
         <v/>
       </c>
-      <c r="N12" s="36" t="inlineStr"/>
+      <c r="N12" s="36" t="n">
+        <v>0.000157</v>
+      </c>
       <c r="O12" s="15" t="inlineStr">
         <is>
-          <t>Runs across portfolio to detect risk/opportunity changes.</t>
+          <t>Measured (5 runs, n=90 calls): Haiku 4.5, avg in=531 out=129. Real Anthropic API.</t>
         </is>
       </c>
     </row>
@@ -1099,10 +1101,10 @@
         <v>750</v>
       </c>
       <c r="E13" s="35" t="n">
+        <v>2504</v>
+      </c>
+      <c r="F13" s="35" t="n">
         <v>800</v>
-      </c>
-      <c r="F13" s="35" t="n">
-        <v>250</v>
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
@@ -1135,10 +1137,12 @@
         <f>IF(L13="","",L13*260)</f>
         <v/>
       </c>
-      <c r="N13" s="36" t="inlineStr"/>
+      <c r="N13" s="36" t="n">
+        <v>0.004564</v>
+      </c>
       <c r="O13" s="15" t="inlineStr">
         <is>
-          <t>Ranks accounts needing attention today.</t>
+          <t>Measured (5 runs, n=5): Sonnet 4.6, 1 call/run synthesising 18 reviews. Note: at 750-account scale would shift to hierarchical (per-segment then per-account) to avoid attention dilution.</t>
         </is>
       </c>
     </row>
@@ -1162,10 +1166,10 @@
         <v>6</v>
       </c>
       <c r="E14" s="35" t="n">
-        <v>900</v>
+        <v>576</v>
       </c>
       <c r="F14" s="35" t="n">
-        <v>250</v>
+        <v>145</v>
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
@@ -1198,10 +1202,12 @@
         <f>IF(L14="","",L14*260)</f>
         <v/>
       </c>
-      <c r="N14" s="36" t="inlineStr"/>
+      <c r="N14" s="36" t="n">
+        <v>0.000174</v>
+      </c>
       <c r="O14" s="15" t="inlineStr">
         <is>
-          <t>Assumes ~30 tickets/week = ~6/day.</t>
+          <t>Measured (5 runs, n=60): Haiku 4.5. My impl combines triage + draft response in one call.</t>
         </is>
       </c>
     </row>
@@ -1261,10 +1267,12 @@
         <f>IF(L15="","",L15*260)</f>
         <v/>
       </c>
-      <c r="N15" s="36" t="inlineStr"/>
+      <c r="N15" s="36" t="n">
+        <v>0.000171</v>
+      </c>
       <c r="O15" s="15" t="inlineStr">
         <is>
-          <t>Creates action, response, or escalation recommendation.</t>
+          <t>My impl combines triage + drafting into one Haiku call (row 14). Row 15 unchanged from template default; production might split if response drafting needs Sonnet-quality.</t>
         </is>
       </c>
     </row>
@@ -1288,10 +1296,10 @@
         <v>2.4</v>
       </c>
       <c r="E16" s="35" t="n">
-        <v>2500</v>
+        <v>625</v>
       </c>
       <c r="F16" s="35" t="n">
-        <v>800</v>
+        <v>776</v>
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
@@ -1324,10 +1332,12 @@
         <f>IF(L16="","",L16*260)</f>
         <v/>
       </c>
-      <c r="N16" s="36" t="inlineStr"/>
+      <c r="N16" s="36" t="n">
+        <v>0.002986</v>
+      </c>
       <c r="O16" s="15" t="inlineStr">
         <is>
-          <t>Assumes ~12 check-ins/week = ~2.4/day.</t>
+          <t>Measured (5 runs, n=60): Sonnet 4.6, full brief with carry-forward of open follow-ups. Codex review flag: routine check-ins could route to Haiku conditionally on health/value triggers.</t>
         </is>
       </c>
     </row>
@@ -1351,10 +1361,10 @@
         <v>2.4</v>
       </c>
       <c r="E17" s="35" t="n">
-        <v>2200</v>
+        <v>625</v>
       </c>
       <c r="F17" s="35" t="n">
-        <v>700</v>
+        <v>776</v>
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
@@ -1387,10 +1397,12 @@
         <f>IF(L17="","",L17*260)</f>
         <v/>
       </c>
-      <c r="N17" s="36" t="inlineStr"/>
+      <c r="N17" s="36" t="n">
+        <v>0.002986</v>
+      </c>
       <c r="O17" s="15" t="inlineStr">
         <is>
-          <t>Uses prior notes and account state for next steps.</t>
+          <t>Not separately measured this build; same pattern + cost shape as checkin_prep (row 16).</t>
         </is>
       </c>
     </row>
@@ -1414,10 +1426,10 @@
         <v>20</v>
       </c>
       <c r="E18" s="35" t="n">
-        <v>1600</v>
+        <v>653</v>
       </c>
       <c r="F18" s="35" t="n">
-        <v>450</v>
+        <v>781</v>
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
@@ -1450,10 +1462,12 @@
         <f>IF(L18="","",L18*260)</f>
         <v/>
       </c>
-      <c r="N18" s="36" t="inlineStr"/>
+      <c r="N18" s="36" t="n">
+        <v>0.003024</v>
+      </c>
       <c r="O18" s="15" t="inlineStr">
         <is>
-          <t>Reviews junior/system outputs against standards.</t>
+          <t>Measured (5 runs, n=40): Sonnet 4.6 generator-side review.</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1530,7 @@
       <c r="N19" s="36" t="inlineStr"/>
       <c r="O19" s="15" t="inlineStr">
         <is>
-          <t>Detects common underperformance patterns by segment.</t>
+          <t>Deterministic Python detector in my impl; no LLM cost. Cost shown is template default for an LLM-detector design alternative.</t>
         </is>
       </c>
     </row>
@@ -1540,10 +1554,10 @@
         <v>5</v>
       </c>
       <c r="E20" s="35" t="n">
-        <v>3500</v>
+        <v>1487</v>
       </c>
       <c r="F20" s="35" t="n">
-        <v>1200</v>
+        <v>834</v>
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
@@ -1576,10 +1590,12 @@
         <f>IF(L20="","",L20*260)</f>
         <v/>
       </c>
-      <c r="N20" s="36" t="inlineStr"/>
+      <c r="N20" s="36" t="n">
+        <v>0.014469</v>
+      </c>
       <c r="O20" s="15" t="inlineStr">
         <is>
-          <t>Designs corrective action and measurement plan.</t>
+          <t>Measured (5 runs, n=5): Opus 4.7. Fires conditionally on segment-level decline; 1 call per run in this dataset.</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1658,7 @@
       <c r="N21" s="36" t="inlineStr"/>
       <c r="O21" s="15" t="inlineStr">
         <is>
-          <t>Routes issue to resolution, follow-up, or escalation path.</t>
+          <t>Not implemented this build. Would map to Haiku-tier triage (~$0.00017/call); production adds webhook intake + SLA clock.</t>
         </is>
       </c>
     </row>
@@ -1705,7 +1721,7 @@
       <c r="N22" s="36" t="inlineStr"/>
       <c r="O22" s="15" t="inlineStr">
         <is>
-          <t>Creates concise packet for human/specialist escalation.</t>
+          <t>Not implemented as separate call; covered by intervention_design when escalation is needed. Production would build a dedicated Sonnet packet per Codex review feedback.</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1784,7 @@
       <c r="N23" s="36" t="inlineStr"/>
       <c r="O23" s="15" t="inlineStr">
         <is>
-          <t>Retrieves relevant prior notes/history.</t>
+          <t>In-process pandas filter; zero LLM cost. Embedding tier (template default) would apply with vector retrieval at scale.</t>
         </is>
       </c>
     </row>
@@ -1792,10 +1808,10 @@
         <v>35</v>
       </c>
       <c r="E24" s="35" t="n">
-        <v>1200</v>
+        <v>1494</v>
       </c>
       <c r="F24" s="35" t="n">
-        <v>250</v>
+        <v>80</v>
       </c>
       <c r="G24" s="15" t="inlineStr">
         <is>
@@ -1828,10 +1844,12 @@
         <f>IF(L24="","",L24*260)</f>
         <v/>
       </c>
-      <c r="N24" s="36" t="inlineStr"/>
+      <c r="N24" s="36" t="n">
+        <v>0.000272</v>
+      </c>
       <c r="O24" s="15" t="inlineStr">
         <is>
-          <t>Checks outputs against quality rules and failure criteria.</t>
+          <t>Measured (5 runs, n=40): Haiku 4.5 INDEPENDENT JUDGE. Different model from Sonnet generator = real discriminator separation. Serves as the automated workflow eval. Known limitation: judge sees first reviewer verdict (anchoring risk); blind-judge variant is the upgrade.</t>
         </is>
       </c>
     </row>

</xml_diff>